<commit_message>
Acertando o calendário SuperLogica
</commit_message>
<xml_diff>
--- a/Calendário de final de semestre - SuperLogica.xlsx
+++ b/Calendário de final de semestre - SuperLogica.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\27120642839\Documents\projetos_documentacao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3CE35F8-8DAB-47BC-8E87-6045ED8DBB1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB282BE8-2412-44F4-B938-F24086B4B1A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="11">
   <si>
     <t>MAIO</t>
   </si>
@@ -66,6 +66,9 @@
   </si>
   <si>
     <t>Entrega documentação TCC (GitHub)</t>
+  </si>
+  <si>
+    <t>Pergunta oral do código</t>
   </si>
 </sst>
 </file>
@@ -96,7 +99,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -139,6 +142,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF00FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -177,42 +186,47 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF00FF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -487,39 +501,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:T9"/>
+  <dimension ref="B2:T10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="18" width="2.85546875" customWidth="1"/>
-    <col min="19" max="19" width="2.85546875" style="14" customWidth="1"/>
-    <col min="20" max="20" width="33.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="2.85546875" style="12" customWidth="1"/>
+    <col min="20" max="20" width="33.5703125" bestFit="1" customWidth="1"/>
     <col min="21" max="36" width="2.85546875" customWidth="1"/>
     <col min="37" max="39" width="3.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="J2" s="5" t="s">
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="J2" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="5"/>
-      <c r="P2" s="5"/>
-      <c r="S2" s="11">
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="17"/>
+      <c r="O2" s="17"/>
+      <c r="P2" s="17"/>
+      <c r="S2" s="9">
         <v>27</v>
       </c>
-      <c r="T2" s="8" t="s">
+      <c r="T2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -566,19 +580,19 @@
       <c r="P3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="S3" s="12"/>
-      <c r="T3" s="9"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="7"/>
     </row>
     <row r="4" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6">
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5">
         <v>1</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="5">
         <f>G4+1</f>
         <v>2</v>
       </c>
@@ -590,121 +604,121 @@
         <f>K4+1</f>
         <v>2</v>
       </c>
-      <c r="M4" s="10">
+      <c r="M4" s="8">
         <f t="shared" ref="M4:P4" si="0">L4+1</f>
         <v>3</v>
       </c>
-      <c r="N4" s="6">
+      <c r="N4" s="5">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="O4" s="6">
+      <c r="O4" s="5">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="P4" s="6">
+      <c r="P4" s="5">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="S4" s="13">
+      <c r="S4" s="11">
         <v>3</v>
       </c>
-      <c r="T4" s="8" t="s">
+      <c r="T4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B5" s="6">
+      <c r="B5" s="5">
         <f>H4+1</f>
         <v>3</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="5">
         <f>B5+1</f>
         <v>4</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="5">
         <f t="shared" ref="D5:H5" si="1">C5+1</f>
         <v>5</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="5">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="5">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="5">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="5">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="J5" s="6">
+      <c r="J5" s="5">
         <f>P4+1</f>
         <v>7</v>
       </c>
-      <c r="K5" s="17">
+      <c r="K5" s="15">
         <f>J5+1</f>
         <v>8</v>
       </c>
-      <c r="L5" s="17">
+      <c r="L5" s="15">
         <f t="shared" ref="L5:P5" si="2">K5+1</f>
         <v>9</v>
       </c>
-      <c r="M5" s="15">
+      <c r="M5" s="13">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="N5" s="17">
+      <c r="N5" s="15">
         <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="O5" s="17">
+      <c r="O5" s="15">
         <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="P5" s="6">
+      <c r="P5" s="5">
         <f t="shared" si="2"/>
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B6" s="6">
+      <c r="B6" s="5">
         <f t="shared" ref="B6:B9" si="3">H5+1</f>
         <v>10</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="5">
         <f t="shared" ref="C6:H6" si="4">B6+1</f>
         <v>11</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="5">
         <f t="shared" si="4"/>
         <v>12</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="5">
         <f t="shared" si="4"/>
         <v>13</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="5">
         <f t="shared" si="4"/>
         <v>14</v>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="5">
         <f t="shared" si="4"/>
         <v>15</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="5">
         <f t="shared" si="4"/>
         <v>16</v>
       </c>
-      <c r="J6" s="6">
-        <f t="shared" ref="J6:J9" si="5">P5+1</f>
+      <c r="J6" s="5">
+        <f t="shared" ref="J6:J8" si="5">P5+1</f>
         <v>14</v>
       </c>
-      <c r="K6" s="17">
+      <c r="K6" s="15">
         <f t="shared" ref="K6:P6" si="6">J6+1</f>
         <v>15</v>
       </c>
@@ -712,7 +726,7 @@
         <f t="shared" si="6"/>
         <v>16</v>
       </c>
-      <c r="M6" s="2">
+      <c r="M6" s="18">
         <f t="shared" si="6"/>
         <v>17</v>
       </c>
@@ -724,27 +738,27 @@
         <f t="shared" si="6"/>
         <v>19</v>
       </c>
-      <c r="P6" s="6">
+      <c r="P6" s="5">
         <f t="shared" si="6"/>
         <v>20</v>
       </c>
-      <c r="S6" s="16">
+      <c r="S6" s="14">
         <v>10</v>
       </c>
-      <c r="T6" s="8" t="s">
+      <c r="T6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B7" s="6">
+      <c r="B7" s="5">
         <f t="shared" si="3"/>
         <v>17</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="5">
         <f t="shared" ref="C7:H7" si="7">B7+1</f>
         <v>18</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="5">
         <f t="shared" si="7"/>
         <v>19</v>
       </c>
@@ -760,11 +774,11 @@
         <f t="shared" si="7"/>
         <v>22</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="5">
         <f t="shared" si="7"/>
         <v>23</v>
       </c>
-      <c r="J7" s="6">
+      <c r="J7" s="5">
         <f t="shared" si="5"/>
         <v>21</v>
       </c>
@@ -772,29 +786,29 @@
         <f t="shared" ref="K7:P7" si="8">J7+1</f>
         <v>22</v>
       </c>
-      <c r="L7" s="6">
+      <c r="L7" s="5">
         <f t="shared" si="8"/>
         <v>23</v>
       </c>
-      <c r="M7" s="6">
+      <c r="M7" s="5">
         <f t="shared" si="8"/>
         <v>24</v>
       </c>
-      <c r="N7" s="6">
+      <c r="N7" s="5">
         <f t="shared" si="8"/>
         <v>25</v>
       </c>
-      <c r="O7" s="6">
+      <c r="O7" s="5">
         <f t="shared" si="8"/>
         <v>26</v>
       </c>
-      <c r="P7" s="6">
+      <c r="P7" s="5">
         <f t="shared" si="8"/>
         <v>27</v>
       </c>
     </row>
     <row r="8" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B8" s="6">
+      <c r="B8" s="5">
         <f t="shared" si="3"/>
         <v>24</v>
       </c>
@@ -806,7 +820,7 @@
         <f t="shared" si="9"/>
         <v>26</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="6">
         <f t="shared" si="9"/>
         <v>27</v>
       </c>
@@ -818,33 +832,33 @@
         <f t="shared" si="9"/>
         <v>29</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="5">
         <f t="shared" si="9"/>
         <v>30</v>
       </c>
-      <c r="J8" s="6">
+      <c r="J8" s="5">
         <f t="shared" si="5"/>
         <v>28</v>
       </c>
-      <c r="K8" s="6">
-        <f t="shared" ref="K8:P8" si="10">J8+1</f>
+      <c r="K8" s="5">
+        <f t="shared" ref="K8:L8" si="10">J8+1</f>
         <v>29</v>
       </c>
-      <c r="L8" s="6">
+      <c r="L8" s="5">
         <f t="shared" si="10"/>
         <v>30</v>
       </c>
-      <c r="M8" s="6"/>
-      <c r="N8" s="6"/>
-      <c r="O8" s="6"/>
-      <c r="P8" s="6"/>
-      <c r="S8" s="18"/>
-      <c r="T8" s="8" t="s">
+      <c r="M8" s="5"/>
+      <c r="N8" s="5"/>
+      <c r="O8" s="5"/>
+      <c r="P8" s="5"/>
+      <c r="S8" s="16"/>
+      <c r="T8" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B9" s="6">
+      <c r="B9" s="5">
         <f t="shared" si="3"/>
         <v>31</v>
       </c>
@@ -854,13 +868,21 @@
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="6"/>
-      <c r="P9" s="6"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
+      <c r="P9" s="5"/>
+    </row>
+    <row r="10" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="S10" s="18">
+        <v>17</v>
+      </c>
+      <c r="T10" t="s">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>